<commit_message>
Update CapitalRemittancePayments sample document as it had incorrect xl cell validation on folio no (#1749)
</commit_message>
<xml_diff>
--- a/public/sample_uploads/capital_remittance_payments.xlsx
+++ b/public/sample_uploads/capital_remittance_payments.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aseem Karmali\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Khushali\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60BEA56F-EC1D-4B01-8F36-2BDBD657062E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56F2EC4-06BB-49F7-9435-835F8B54D36B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CapitalRemittance" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -541,25 +541,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.4375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.6875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.4140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="7" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="10.375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6875" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" style="1" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.3125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="18.6875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.6640625" style="1" customWidth="1"/>
     <col min="10" max="10" width="11.75" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.3125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="8.625" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.625" style="1"/>
+    <col min="11" max="11" width="13.33203125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.08203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="8.58203125" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.58203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="4" customFormat="1" ht="29.65" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" s="4" customFormat="1" ht="29.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -597,7 +597,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -626,7 +626,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -655,7 +655,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -684,7 +684,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -713,7 +713,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -742,12 +742,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="7" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C187 L2:L1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{EB2EF399-F90C-4B82-BF2F-33FF923BD0C2}">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>